<commit_message>
correct errors reported by Liu
</commit_message>
<xml_diff>
--- a/data/C0003/C0003R03_PARK25_LC_1D_SCAN.xlsx
+++ b/data/C0003/C0003R03_PARK25_LC_1D_SCAN.xlsx
@@ -639,13 +639,13 @@
         <v>37.38822920264325</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>2.8203186408</v>
+        <v>0.7935129599999999</v>
       </c>
       <c r="M2" s="4" t="n">
         <v>0.1454891911560698</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>2.96580783195607</v>
+        <v>0.9390021511560698</v>
       </c>
       <c r="O2" s="4" t="n">
         <v>36.34894575681116</v>
@@ -716,13 +716,13 @@
         <v>38.37212997113386</v>
       </c>
       <c r="L3" s="4" t="n">
-        <v>2.8945375524</v>
+        <v>0.8143948799999998</v>
       </c>
       <c r="M3" s="4" t="n">
         <v>0.1493178540812296</v>
       </c>
       <c r="N3" s="4" t="n">
-        <v>3.04385540648123</v>
+        <v>0.9637127340812294</v>
       </c>
       <c r="O3" s="4" t="n">
         <v>36.27565204541914</v>
@@ -793,13 +793,13 @@
         <v>39.35603073962447</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>2.968756464</v>
+        <v>0.8352767999999999</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>0.1531465170063893</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>3.121902981006389</v>
+        <v>0.9884233170063892</v>
       </c>
       <c r="O4" s="4" t="n">
         <v>36.20505206914466</v>
@@ -870,13 +870,13 @@
         <v>40.33993150811509</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>3.0429753756</v>
+        <v>0.85615872</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>0.156975179931549</v>
+        <v>0.1569751799315491</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>3.199950555531549</v>
+        <v>1.013133899931549</v>
       </c>
       <c r="O5" s="4" t="n">
         <v>36.13699005609593</v>
@@ -947,13 +947,13 @@
         <v>41.3238322766057</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>3.1171942872</v>
+        <v>0.8770406399999998</v>
       </c>
       <c r="M6" s="4" t="n">
         <v>0.1608038428567088</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>3.277998130056709</v>
+        <v>1.037844482856709</v>
       </c>
       <c r="O6" s="4" t="n">
         <v>36.07132214935912</v>
@@ -1024,13 +1024,13 @@
         <v>12.75949324031593</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>3.426209181</v>
+        <v>0.8927020799999998</v>
       </c>
       <c r="M7" s="4" t="n">
         <v>0.2182337867341048</v>
       </c>
       <c r="N7" s="4" t="n">
-        <v>3.644442967734105</v>
+        <v>1.110935866734104</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>37.09968453403143</v>
@@ -1101,13 +1101,13 @@
         <v>13.09526937821899</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>3.5163725805</v>
+        <v>0.9161942399999999</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>0.2239767811218444</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>3.740349361621844</v>
+        <v>1.140171021121844</v>
       </c>
       <c r="O8" s="4" t="n">
         <v>37.01798281068388</v>
@@ -1178,13 +1178,13 @@
         <v>13.43104551612204</v>
       </c>
       <c r="L9" s="4" t="n">
-        <v>3.606535980000001</v>
+        <v>0.9396864</v>
       </c>
       <c r="M9" s="4" t="n">
         <v>0.229719775509584</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>3.836255755509585</v>
+        <v>1.169406175509584</v>
       </c>
       <c r="O9" s="4" t="n">
         <v>36.93918479590487</v>
@@ -1255,13 +1255,13 @@
         <v>13.76682165402508</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>3.6966993795</v>
+        <v>0.96317856</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>0.2354627698973235</v>
+        <v>0.2354627698973236</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>3.932162149397324</v>
+        <v>1.198641329897324</v>
       </c>
       <c r="O10" s="4" t="n">
         <v>36.86312870706875</v>
@@ -1332,13 +1332,13 @@
         <v>14.10259779192814</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>3.786862779</v>
+        <v>0.98667072</v>
       </c>
       <c r="M11" s="4" t="n">
         <v>0.2412057642850631</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>4.028068543285063</v>
+        <v>1.227876484285063</v>
       </c>
       <c r="O11" s="4" t="n">
         <v>36.78966501712407</v>
@@ -1409,13 +1409,13 @@
         <v>6.285672978218058</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4.0320997212</v>
+        <v>0.9918912</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>0.2909783823121397</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>4.32307810351214</v>
+        <v>1.28286958231214</v>
       </c>
       <c r="O12" s="4" t="n">
         <v>37.5252488245417</v>
@@ -1486,13 +1486,13 @@
         <v>6.451085425013272</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>4.1382076086</v>
+        <v>1.0179936</v>
       </c>
       <c r="M13" s="4" t="n">
         <v>0.2986357081624592</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>4.436843316762459</v>
+        <v>1.316629308162459</v>
       </c>
       <c r="O13" s="4" t="n">
         <v>37.43920889238697</v>
@@ -1563,13 +1563,13 @@
         <v>6.616497871808482</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>4.244315496</v>
+        <v>1.044096</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>0.3062930340127786</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>4.550608530012779</v>
+        <v>1.350389034012779</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>37.35616863191719</v>
@@ -1640,13 +1640,13 @@
         <v>6.781910318603694</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>4.3504233834</v>
+        <v>1.0701984</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.313950359863098</v>
+        <v>0.3139503598630981</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>4.664373743263098</v>
+        <v>1.384148759863098</v>
       </c>
       <c r="O15" s="4" t="n">
         <v>37.27596258856259</v>
@@ -1717,13 +1717,13 @@
         <v>6.947322765398907</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>4.456531270800001</v>
+        <v>1.0963008</v>
       </c>
       <c r="M16" s="4" t="n">
         <v>0.3216076857134175</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>4.778138956513419</v>
+        <v>1.417908485713417</v>
       </c>
       <c r="O16" s="4" t="n">
         <v>37.19843800541032</v>
@@ -1794,13 +1794,13 @@
         <v>3.793249021129413</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>4.637990261400001</v>
+        <v>1.09108032</v>
       </c>
       <c r="M17" s="4" t="n">
         <v>0.3637229778901746</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>5.001713239290175</v>
+        <v>1.454803297890175</v>
       </c>
       <c r="O17" s="4" t="n">
         <v>37.70011226652623</v>
@@ -1871,13 +1871,13 @@
         <v>3.893071363790714</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>4.7600426367</v>
+        <v>1.11979296</v>
       </c>
       <c r="M18" s="4" t="n">
         <v>0.373294635203074</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>5.133337271903073</v>
+        <v>1.493087595203074</v>
       </c>
       <c r="O18" s="4" t="n">
         <v>37.61237230758533</v>
@@ -1948,13 +1948,13 @@
         <v>3.992893706452014</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>4.882095012000001</v>
+        <v>1.1485056</v>
       </c>
       <c r="M19" s="4" t="n">
         <v>0.3828662925159733</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>5.264961304515974</v>
+        <v>1.531371892515973</v>
       </c>
       <c r="O19" s="4" t="n">
         <v>37.52766933246858</v>
@@ -2025,13 +2025,13 @@
         <v>4.092716049113315</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>5.0041473873</v>
+        <v>1.17721824</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>0.3924379498288725</v>
+        <v>0.3924379498288726</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>5.396585337128872</v>
+        <v>1.569656189828873</v>
       </c>
       <c r="O20" s="4" t="n">
         <v>37.44583605908487</v>
@@ -2102,13 +2102,13 @@
         <v>4.192538391774614</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>5.126199762600001</v>
+        <v>1.20593088</v>
       </c>
       <c r="M21" s="4" t="n">
         <v>0.4020096071417719</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>5.528209369741773</v>
+        <v>1.607940487141772</v>
       </c>
       <c r="O21" s="4" t="n">
         <v>37.36671814683267</v>
@@ -2179,13 +2179,13 @@
         <v>30.8701982756164</v>
       </c>
       <c r="L22" s="4" t="n">
-        <v>2.8864447208</v>
+        <v>0.72738688</v>
       </c>
       <c r="M22" s="4" t="n">
         <v>0.1697373896820815</v>
       </c>
       <c r="N22" s="4" t="n">
-        <v>3.056182110482081</v>
+        <v>0.8971242696820814</v>
       </c>
       <c r="O22" s="4" t="n">
         <v>36.04842390714253</v>
@@ -2256,13 +2256,13 @@
         <v>31.68257191444841</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>2.9624037924</v>
+        <v>0.74652864</v>
       </c>
       <c r="M23" s="4" t="n">
         <v>0.1742041630947678</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>3.136607955494768</v>
+        <v>0.9207328030947678</v>
       </c>
       <c r="O23" s="4" t="n">
         <v>35.97874905945248</v>
@@ -2333,13 +2333,13 @@
         <v>32.49494555328042</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>3.038362864</v>
+        <v>0.7656703999999999</v>
       </c>
       <c r="M24" s="4" t="n">
         <v>0.1786709365074542</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>3.217033800507454</v>
+        <v>0.944341336507454</v>
       </c>
       <c r="O24" s="4" t="n">
         <v>35.9116620989638</v>
@@ -2410,13 +2410,13 @@
         <v>33.30731919211243</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>3.1143219356</v>
+        <v>0.7848121600000002</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>0.1831377099201405</v>
+        <v>0.1831377099201406</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>3.29745964552014</v>
+        <v>0.9679498699201408</v>
       </c>
       <c r="O25" s="4" t="n">
         <v>35.84701059020399</v>
@@ -2487,13 +2487,13 @@
         <v>34.11969283094444</v>
       </c>
       <c r="L26" s="4" t="n">
-        <v>3.1902810072</v>
+        <v>0.8039539199999998</v>
       </c>
       <c r="M26" s="4" t="n">
         <v>0.1876044833328269</v>
       </c>
       <c r="N26" s="4" t="n">
-        <v>3.377885490532827</v>
+        <v>0.9915584033328266</v>
       </c>
       <c r="O26" s="4" t="n">
         <v>35.78465394070306</v>
@@ -2564,13 +2564,13 @@
         <v>10.27458113958557</v>
       </c>
       <c r="L27" s="4" t="n">
-        <v>3.492335261</v>
+        <v>0.7935129599999998</v>
       </c>
       <c r="M27" s="4" t="n">
         <v>0.2546060845231223</v>
       </c>
       <c r="N27" s="4" t="n">
-        <v>3.746941345523122</v>
+        <v>1.048119044523122</v>
       </c>
       <c r="O27" s="4" t="n">
         <v>36.82013020646833</v>
@@ -2641,13 +2641,13 @@
         <v>10.54496485378519</v>
       </c>
       <c r="L28" s="4" t="n">
-        <v>3.5842388205</v>
+        <v>0.8143948799999998</v>
       </c>
       <c r="M28" s="4" t="n">
         <v>0.2613062446421518</v>
       </c>
       <c r="N28" s="4" t="n">
-        <v>3.845545065142152</v>
+        <v>1.075701124642152</v>
       </c>
       <c r="O28" s="4" t="n">
         <v>36.74144603556452</v>
@@ -2718,13 +2718,13 @@
         <v>10.81534856798481</v>
       </c>
       <c r="L29" s="4" t="n">
-        <v>3.67614238</v>
+        <v>0.8352767999999999</v>
       </c>
       <c r="M29" s="4" t="n">
         <v>0.2680064047611813</v>
       </c>
       <c r="N29" s="4" t="n">
-        <v>3.944148784761181</v>
+        <v>1.103283204761181</v>
       </c>
       <c r="O29" s="4" t="n">
         <v>36.66559513730225</v>
@@ -2795,13 +2795,13 @@
         <v>11.08573228218443</v>
       </c>
       <c r="L30" s="4" t="n">
-        <v>3.768045939499999</v>
+        <v>0.8561587199999999</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>0.2747065648802108</v>
+        <v>0.2747065648802109</v>
       </c>
       <c r="N30" s="4" t="n">
-        <v>4.042752504380211</v>
+        <v>1.130865284880211</v>
       </c>
       <c r="O30" s="4" t="n">
         <v>36.59241783270686</v>
@@ -2872,13 +2872,13 @@
         <v>11.35611599638405</v>
       </c>
       <c r="L31" s="4" t="n">
-        <v>3.859949498999999</v>
+        <v>0.8770406399999998</v>
       </c>
       <c r="M31" s="4" t="n">
         <v>0.2814067249992404</v>
       </c>
       <c r="N31" s="4" t="n">
-        <v>4.14135622399924</v>
+        <v>1.15844736499924</v>
       </c>
       <c r="O31" s="4" t="n">
         <v>36.52176651902938</v>
@@ -2949,13 +2949,13 @@
         <v>4.92373647512472</v>
       </c>
       <c r="L32" s="4" t="n">
-        <v>4.0982258012</v>
+        <v>0.85963904</v>
       </c>
       <c r="M32" s="4" t="n">
         <v>0.3394747793641629</v>
       </c>
       <c r="N32" s="4" t="n">
-        <v>4.437700580564163</v>
+        <v>1.199113819364163</v>
       </c>
       <c r="O32" s="4" t="n">
         <v>37.31508226699245</v>
@@ -3026,13 +3026,13 @@
         <v>5.053308487628003</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>4.2060738486</v>
+        <v>0.8822611199999998</v>
       </c>
       <c r="M33" s="4" t="n">
         <v>0.3484083261895357</v>
       </c>
       <c r="N33" s="4" t="n">
-        <v>4.554482174789536</v>
+        <v>1.230669446189535</v>
       </c>
       <c r="O33" s="4" t="n">
         <v>37.23114753870869</v>
@@ -3103,13 +3103,13 @@
         <v>5.182880500131284</v>
       </c>
       <c r="L34" s="4" t="n">
-        <v>4.313921896</v>
+        <v>0.9048831999999999</v>
       </c>
       <c r="M34" s="4" t="n">
         <v>0.3573418730149084</v>
       </c>
       <c r="N34" s="4" t="n">
-        <v>4.671263769014908</v>
+        <v>1.262225073014908</v>
       </c>
       <c r="O34" s="4" t="n">
         <v>37.15016634742845</v>
@@ -3180,13 +3180,13 @@
         <v>5.312452512634566</v>
       </c>
       <c r="L35" s="4" t="n">
-        <v>4.421769943399999</v>
+        <v>0.9275052800000001</v>
       </c>
       <c r="M35" s="4" t="n">
         <v>0.3662754198402811</v>
       </c>
       <c r="N35" s="4" t="n">
-        <v>4.78804536324028</v>
+        <v>1.293780699840281</v>
       </c>
       <c r="O35" s="4" t="n">
         <v>37.07197516432142</v>
@@ -3257,13 +3257,13 @@
         <v>5.442024525137849</v>
       </c>
       <c r="L36" s="4" t="n">
-        <v>4.529617990799999</v>
+        <v>0.9501273599999998</v>
       </c>
       <c r="M36" s="4" t="n">
         <v>0.3752089666656538</v>
       </c>
       <c r="N36" s="4" t="n">
-        <v>4.904826957465653</v>
+        <v>1.325336326665653</v>
       </c>
       <c r="O36" s="4" t="n">
         <v>36.99642291298903</v>
@@ -3334,13 +3334,13 @@
         <v>2.889083587839437</v>
       </c>
       <c r="L37" s="4" t="n">
-        <v>4.704116341400001</v>
+        <v>0.92576512</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>0.4243434742052037</v>
       </c>
       <c r="N37" s="4" t="n">
-        <v>5.128459815605204</v>
+        <v>1.350108594205204</v>
       </c>
       <c r="O37" s="4" t="n">
         <v>37.59355196100468</v>
@@ -3411,13 +3411,13 @@
         <v>2.965112103308897</v>
       </c>
       <c r="L38" s="4" t="n">
-        <v>4.8279088767</v>
+        <v>0.9501273599999996</v>
       </c>
       <c r="M38" s="4" t="n">
         <v>0.4355104077369196</v>
       </c>
       <c r="N38" s="4" t="n">
-        <v>5.26341928443692</v>
+        <v>1.385637767736919</v>
       </c>
       <c r="O38" s="4" t="n">
         <v>37.50684263927545</v>
@@ -3488,13 +3488,13 @@
         <v>3.041140618778356</v>
       </c>
       <c r="L39" s="4" t="n">
-        <v>4.951701411999999</v>
+        <v>0.9744895999999998</v>
       </c>
       <c r="M39" s="4" t="n">
         <v>0.4466773412686355</v>
       </c>
       <c r="N39" s="4" t="n">
-        <v>5.398378753268635</v>
+        <v>1.421166941268635</v>
       </c>
       <c r="O39" s="4" t="n">
         <v>37.42314764057592</v>
@@ -3565,13 +3565,13 @@
         <v>3.117169134247814</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>5.075493947299999</v>
+        <v>0.9988518399999998</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>0.4578442748003513</v>
+        <v>0.4578442748003514</v>
       </c>
       <c r="N40" s="4" t="n">
-        <v>5.53333822210035</v>
+        <v>1.456696114800351</v>
       </c>
       <c r="O40" s="4" t="n">
         <v>37.34230082325222</v>
@@ -3642,13 +3642,13 @@
         <v>3.193197649717274</v>
       </c>
       <c r="L41" s="4" t="n">
-        <v>5.199286482599998</v>
+        <v>1.02321408</v>
       </c>
       <c r="M41" s="4" t="n">
         <v>0.4690112083320673</v>
       </c>
       <c r="N41" s="4" t="n">
-        <v>5.668297690932065</v>
+        <v>1.492225288332067</v>
       </c>
       <c r="O41" s="4" t="n">
         <v>37.26414883433036</v>
@@ -3719,13 +3719,13 @@
         <v>26.28774851780796</v>
       </c>
       <c r="L42" s="4" t="n">
-        <v>2.9525708008</v>
+        <v>0.6653936800000002</v>
       </c>
       <c r="M42" s="4" t="n">
         <v>0.1939855882080931</v>
       </c>
       <c r="N42" s="4" t="n">
-        <v>3.146556389008093</v>
+        <v>0.8593792682080933</v>
       </c>
       <c r="O42" s="4" t="n">
         <v>35.78878170815381</v>
@@ -3796,13 +3796,13 @@
         <v>26.97953137353975</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>3.0302700324</v>
+        <v>0.6829040400000003</v>
       </c>
       <c r="M43" s="4" t="n">
         <v>0.1990904721083061</v>
       </c>
       <c r="N43" s="4" t="n">
-        <v>3.229360504508306</v>
+        <v>0.8819945121083064</v>
       </c>
       <c r="O43" s="4" t="n">
         <v>35.72232334625234</v>
@@ -3873,13 +3873,13 @@
         <v>27.67131422927154</v>
       </c>
       <c r="L44" s="4" t="n">
-        <v>3.107969264</v>
+        <v>0.7004144000000002</v>
       </c>
       <c r="M44" s="4" t="n">
         <v>0.2041953560085191</v>
       </c>
       <c r="N44" s="4" t="n">
-        <v>3.312164620008519</v>
+        <v>0.9046097560085193</v>
       </c>
       <c r="O44" s="4" t="n">
         <v>35.6583500371619</v>
@@ -3950,13 +3950,13 @@
         <v>28.36309708500332</v>
       </c>
       <c r="L45" s="4" t="n">
-        <v>3.1856684956</v>
+        <v>0.7179247600000003</v>
       </c>
       <c r="M45" s="4" t="n">
         <v>0.209300239908732</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>3.394968735508732</v>
+        <v>0.9272249999087323</v>
       </c>
       <c r="O45" s="4" t="n">
         <v>35.59671311171307</v>
@@ -4027,13 +4027,13 @@
         <v>29.05487994073511</v>
       </c>
       <c r="L46" s="4" t="n">
-        <v>3.2633677272</v>
+        <v>0.7354351200000003</v>
       </c>
       <c r="M46" s="4" t="n">
         <v>0.214405123808945</v>
       </c>
       <c r="N46" s="4" t="n">
-        <v>3.477772851008945</v>
+        <v>0.9498402438089453</v>
       </c>
       <c r="O46" s="4" t="n">
         <v>35.53727565155639</v>
@@ -4104,13 +4104,13 @@
         <v>8.594589283295882</v>
       </c>
       <c r="L47" s="4" t="n">
-        <v>3.558461341</v>
+        <v>0.6994899400000001</v>
       </c>
       <c r="M47" s="4" t="n">
         <v>0.2909783823121397</v>
       </c>
       <c r="N47" s="4" t="n">
-        <v>3.849439723312139</v>
+        <v>0.9904683223121398</v>
       </c>
       <c r="O47" s="4" t="n">
         <v>36.56677983174237</v>
@@ -4181,13 +4181,13 @@
         <v>8.82076268548788</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>3.6521050605</v>
+        <v>0.7178975700000003</v>
       </c>
       <c r="M48" s="4" t="n">
         <v>0.2986357081624592</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>3.95074076866246</v>
+        <v>1.016533278162459</v>
       </c>
       <c r="O48" s="4" t="n">
         <v>36.49094788486686</v>
@@ -4258,13 +4258,13 @@
         <v>9.046936087679876</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>3.74574878</v>
+        <v>0.7363052000000003</v>
       </c>
       <c r="M49" s="4" t="n">
         <v>0.3062930340127786</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>4.052041814012779</v>
+        <v>1.042598234012779</v>
       </c>
       <c r="O49" s="4" t="n">
         <v>36.41787788959546</v>
@@ -4335,13 +4335,13 @@
         <v>9.273109489871873</v>
       </c>
       <c r="L50" s="4" t="n">
-        <v>3.8393924995</v>
+        <v>0.7547128300000002</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>0.313950359863098</v>
+        <v>0.3139503598630981</v>
       </c>
       <c r="N50" s="4" t="n">
-        <v>4.153342859363097</v>
+        <v>1.068663189863098</v>
       </c>
       <c r="O50" s="4" t="n">
         <v>36.34741213892779</v>
@@ -4412,13 +4412,13 @@
         <v>9.499282892063869</v>
       </c>
       <c r="L51" s="4" t="n">
-        <v>3.933036219</v>
+        <v>0.7731204600000001</v>
       </c>
       <c r="M51" s="4" t="n">
         <v>0.3216076857134175</v>
       </c>
       <c r="N51" s="4" t="n">
-        <v>4.254643904713418</v>
+        <v>1.094728145713418</v>
       </c>
       <c r="O51" s="4" t="n">
         <v>36.27940489974429</v>
@@ -4489,13 +4489,13 @@
         <v>4.037183408068714</v>
       </c>
       <c r="L52" s="4" t="n">
-        <v>4.1643518812</v>
+        <v>0.7335862000000004</v>
       </c>
       <c r="M52" s="4" t="n">
         <v>0.3879711764161862</v>
       </c>
       <c r="N52" s="4" t="n">
-        <v>4.552323057616186</v>
+        <v>1.121557376416187</v>
       </c>
       <c r="O52" s="4" t="n">
         <v>37.09432830369191</v>
@@ -4566,13 +4566,13 @@
         <v>4.143425076702101</v>
       </c>
       <c r="L53" s="4" t="n">
-        <v>4.273940088600001</v>
+        <v>0.7528911000000005</v>
       </c>
       <c r="M53" s="4" t="n">
         <v>0.3981809442166122</v>
       </c>
       <c r="N53" s="4" t="n">
-        <v>4.672121032816613</v>
+        <v>1.151072044216613</v>
       </c>
       <c r="O53" s="4" t="n">
         <v>37.01268311632313</v>
@@ -4643,13 +4643,13 @@
         <v>4.249666745335488</v>
       </c>
       <c r="L54" s="4" t="n">
-        <v>4.383528296000001</v>
+        <v>0.7721960000000004</v>
       </c>
       <c r="M54" s="4" t="n">
         <v>0.4083907120170381</v>
       </c>
       <c r="N54" s="4" t="n">
-        <v>4.79191900801704</v>
+        <v>1.180586712017039</v>
       </c>
       <c r="O54" s="4" t="n">
         <v>36.93394035547854</v>
@@ -4720,13 +4720,13 @@
         <v>4.355908413968876</v>
       </c>
       <c r="L55" s="4" t="n">
-        <v>4.4931165034</v>
+        <v>0.7915009000000005</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>0.418600479817464</v>
+        <v>0.4186004798174641</v>
       </c>
       <c r="N55" s="4" t="n">
-        <v>4.911716983217463</v>
+        <v>1.210101379817464</v>
       </c>
       <c r="O55" s="4" t="n">
         <v>36.85793827990386</v>
@@ -4797,13 +4797,13 @@
         <v>4.462150082602262</v>
       </c>
       <c r="L56" s="4" t="n">
-        <v>4.6027047108</v>
+        <v>0.8108058000000004</v>
       </c>
       <c r="M56" s="4" t="n">
         <v>0.42881024761789</v>
       </c>
       <c r="N56" s="4" t="n">
-        <v>5.03151495841789</v>
+        <v>1.23961604761789</v>
       </c>
       <c r="O56" s="4" t="n">
         <v>36.78452739970628</v>
@@ -4874,13 +4874,13 @@
         <v>2.319441231398063</v>
       </c>
       <c r="L57" s="4" t="n">
-        <v>4.7702424214</v>
+        <v>0.7676824600000001</v>
       </c>
       <c r="M57" s="4" t="n">
         <v>0.4849639705202328</v>
       </c>
       <c r="N57" s="4" t="n">
-        <v>5.255206391920233</v>
+        <v>1.252646430520233</v>
       </c>
       <c r="O57" s="4" t="n">
         <v>37.44137288334456</v>
@@ -4951,13 +4951,13 @@
         <v>2.380479158540118</v>
       </c>
       <c r="L58" s="4" t="n">
-        <v>4.8957751167</v>
+        <v>0.7878846300000002</v>
       </c>
       <c r="M58" s="4" t="n">
         <v>0.4977261802707653</v>
       </c>
       <c r="N58" s="4" t="n">
-        <v>5.393501296970766</v>
+        <v>1.285610810270766</v>
       </c>
       <c r="O58" s="4" t="n">
         <v>37.35616471739561</v>
@@ -5028,13 +5028,13 @@
         <v>2.441517085682172</v>
       </c>
       <c r="L59" s="4" t="n">
-        <v>5.021307812000001</v>
+        <v>0.8080868000000002</v>
       </c>
       <c r="M59" s="4" t="n">
         <v>0.5104883900212978</v>
       </c>
       <c r="N59" s="4" t="n">
-        <v>5.531796202021298</v>
+        <v>1.318575190021298</v>
       </c>
       <c r="O59" s="4" t="n">
         <v>37.2739380332839</v>
@@ -5105,13 +5105,13 @@
         <v>2.502555012824227</v>
       </c>
       <c r="L60" s="4" t="n">
-        <v>5.146840507299999</v>
+        <v>0.8282889700000005</v>
       </c>
       <c r="M60" s="4" t="n">
-        <v>0.5232505997718301</v>
+        <v>0.5232505997718302</v>
       </c>
       <c r="N60" s="4" t="n">
-        <v>5.67009110707183</v>
+        <v>1.351539569771831</v>
       </c>
       <c r="O60" s="4" t="n">
         <v>37.19452817695417</v>
@@ -5182,13 +5182,13 @@
         <v>2.563592939966281</v>
       </c>
       <c r="L61" s="4" t="n">
-        <v>5.2723732026</v>
+        <v>0.8484911400000001</v>
       </c>
       <c r="M61" s="4" t="n">
         <v>0.5360128095223626</v>
       </c>
       <c r="N61" s="4" t="n">
-        <v>5.808386012122362</v>
+        <v>1.384503949522363</v>
       </c>
       <c r="O61" s="4" t="n">
         <v>37.11778308779611</v>
@@ -5259,13 +5259,13 @@
         <v>22.89066508111284</v>
       </c>
       <c r="L62" s="4" t="n">
-        <v>3.0186968808</v>
+        <v>0.7315197600000001</v>
       </c>
       <c r="M62" s="4" t="n">
         <v>0.2182337867341048</v>
       </c>
       <c r="N62" s="4" t="n">
-        <v>3.236930667534105</v>
+        <v>0.9497535467341049</v>
       </c>
       <c r="O62" s="4" t="n">
         <v>35.56198952899148</v>
@@ -5336,13 +5336,13 @@
         <v>23.49305100430002</v>
       </c>
       <c r="L63" s="4" t="n">
-        <v>3.0981362724</v>
+        <v>0.7507702799999998</v>
       </c>
       <c r="M63" s="4" t="n">
-        <v>0.2239767811218444</v>
+        <v>0.2239767811218445</v>
       </c>
       <c r="N63" s="4" t="n">
-        <v>3.322113053521845</v>
+        <v>0.9747470611218443</v>
       </c>
       <c r="O63" s="4" t="n">
         <v>35.49838927456912</v>
@@ -5413,13 +5413,13 @@
         <v>24.0954369274872</v>
       </c>
       <c r="L64" s="4" t="n">
-        <v>3.177575664</v>
+        <v>0.7700208000000002</v>
       </c>
       <c r="M64" s="4" t="n">
-        <v>0.229719775509584</v>
+        <v>0.2297197755095841</v>
       </c>
       <c r="N64" s="4" t="n">
-        <v>3.407295439509584</v>
+        <v>0.9997405755095843</v>
       </c>
       <c r="O64" s="4" t="n">
         <v>35.4371760008792</v>
@@ -5490,13 +5490,13 @@
         <v>24.69782285067438</v>
       </c>
       <c r="L65" s="4" t="n">
-        <v>3.2570150556</v>
+        <v>0.7892713199999999</v>
       </c>
       <c r="M65" s="4" t="n">
-        <v>0.2354627698973236</v>
+        <v>0.2354627698973237</v>
       </c>
       <c r="N65" s="4" t="n">
-        <v>3.492477825497323</v>
+        <v>1.024734089897324</v>
       </c>
       <c r="O65" s="4" t="n">
         <v>35.37820515480708</v>
@@ -5567,13 +5567,13 @@
         <v>25.30020877386156</v>
       </c>
       <c r="L66" s="4" t="n">
-        <v>3.3364544472</v>
+        <v>0.8085218399999999</v>
       </c>
       <c r="M66" s="4" t="n">
         <v>0.2412057642850632</v>
       </c>
       <c r="N66" s="4" t="n">
-        <v>3.577660211485063</v>
+        <v>1.049727604285063</v>
       </c>
       <c r="O66" s="4" t="n">
         <v>35.32134379955687</v>
@@ -5644,13 +5644,13 @@
         <v>7.385329225213477</v>
       </c>
       <c r="L67" s="4" t="n">
-        <v>3.624587421</v>
+        <v>0.7656160200000001</v>
       </c>
       <c r="M67" s="4" t="n">
-        <v>0.3273506801011572</v>
+        <v>0.3273506801011573</v>
       </c>
       <c r="N67" s="4" t="n">
-        <v>3.951938101101157</v>
+        <v>1.092966700101157</v>
       </c>
       <c r="O67" s="4" t="n">
         <v>36.33906133123853</v>
@@ -5721,13 +5721,13 @@
         <v>7.579679994298044</v>
       </c>
       <c r="L68" s="4" t="n">
-        <v>3.719971300500001</v>
+        <v>0.78576381</v>
       </c>
       <c r="M68" s="4" t="n">
-        <v>0.3359651716827666</v>
+        <v>0.3359651716827667</v>
       </c>
       <c r="N68" s="4" t="n">
-        <v>4.055936472182768</v>
+        <v>1.121728981682767</v>
       </c>
       <c r="O68" s="4" t="n">
         <v>36.26588457840234</v>
@@ -5798,13 +5798,13 @@
         <v>7.774030763382609</v>
       </c>
       <c r="L69" s="4" t="n">
-        <v>3.815355180000001</v>
+        <v>0.8059116000000002</v>
       </c>
       <c r="M69" s="4" t="n">
-        <v>0.344579663264376</v>
+        <v>0.3445796632643761</v>
       </c>
       <c r="N69" s="4" t="n">
-        <v>4.159934843264376</v>
+        <v>1.150491263264376</v>
       </c>
       <c r="O69" s="4" t="n">
         <v>36.1953983007955</v>
@@ -5875,13 +5875,13 @@
         <v>7.968381532467173</v>
       </c>
       <c r="L70" s="4" t="n">
-        <v>3.9107390595</v>
+        <v>0.8260593900000002</v>
       </c>
       <c r="M70" s="4" t="n">
-        <v>0.3531941548459854</v>
+        <v>0.3531941548459855</v>
       </c>
       <c r="N70" s="4" t="n">
-        <v>4.263933214345985</v>
+        <v>1.179253544845986</v>
       </c>
       <c r="O70" s="4" t="n">
         <v>36.12744682234457</v>
@@ -5952,13 +5952,13 @@
         <v>8.162732301551737</v>
       </c>
       <c r="L71" s="4" t="n">
-        <v>4.006122938999999</v>
+        <v>0.8462071800000002</v>
       </c>
       <c r="M71" s="4" t="n">
-        <v>0.3618086464275947</v>
+        <v>0.3618086464275948</v>
       </c>
       <c r="N71" s="4" t="n">
-        <v>4.367931585427594</v>
+        <v>1.208015826427595</v>
       </c>
       <c r="O71" s="4" t="n">
         <v>36.06188637962448</v>
@@ -6029,13 +6029,13 @@
         <v>3.417661770324297</v>
       </c>
       <c r="L72" s="4" t="n">
-        <v>4.230477961199999</v>
+        <v>0.7997122799999999</v>
       </c>
       <c r="M72" s="4" t="n">
-        <v>0.4364675734682096</v>
+        <v>0.4364675734682097</v>
       </c>
       <c r="N72" s="4" t="n">
-        <v>4.666945534668208</v>
+        <v>1.23617985346821</v>
       </c>
       <c r="O72" s="4" t="n">
         <v>36.88242885858186</v>
@@ -6106,13 +6106,13 @@
         <v>3.50760023796441</v>
       </c>
       <c r="L73" s="4" t="n">
-        <v>4.341806328600001</v>
+        <v>0.82075734</v>
       </c>
       <c r="M73" s="4" t="n">
-        <v>0.4479535622436888</v>
+        <v>0.4479535622436889</v>
       </c>
       <c r="N73" s="4" t="n">
-        <v>4.78975989084369</v>
+        <v>1.268710902243689</v>
       </c>
       <c r="O73" s="4" t="n">
         <v>36.80306038605933</v>
@@ -6183,13 +6183,13 @@
         <v>3.597538705604523</v>
       </c>
       <c r="L74" s="4" t="n">
-        <v>4.453134696</v>
+        <v>0.8418024000000003</v>
       </c>
       <c r="M74" s="4" t="n">
         <v>0.4594395510191681</v>
       </c>
       <c r="N74" s="4" t="n">
-        <v>4.912574247019168</v>
+        <v>1.301241951019168</v>
       </c>
       <c r="O74" s="4" t="n">
         <v>36.72654155875151</v>
@@ -6260,13 +6260,13 @@
         <v>3.687477173244636</v>
       </c>
       <c r="L75" s="4" t="n">
-        <v>4.564463063400001</v>
+        <v>0.8628474599999998</v>
       </c>
       <c r="M75" s="4" t="n">
-        <v>0.4709255397946472</v>
+        <v>0.4709255397946474</v>
       </c>
       <c r="N75" s="4" t="n">
-        <v>5.035388603194648</v>
+        <v>1.333772999794647</v>
       </c>
       <c r="O75" s="4" t="n">
         <v>36.65271223239366</v>
@@ -6337,13 +6337,13 @@
         <v>3.77741564088475</v>
       </c>
       <c r="L76" s="4" t="n">
-        <v>4.675791430799999</v>
+        <v>0.88389252</v>
       </c>
       <c r="M76" s="4" t="n">
-        <v>0.4824115285701264</v>
+        <v>0.4824115285701265</v>
       </c>
       <c r="N76" s="4" t="n">
-        <v>5.158202959370126</v>
+        <v>1.366304048570127</v>
       </c>
       <c r="O76" s="4" t="n">
         <v>36.58142437213393</v>
@@ -6414,13 +6414,13 @@
         <v>1.932233815432886</v>
       </c>
       <c r="L77" s="4" t="n">
-        <v>4.8363685014</v>
+        <v>0.8338085399999998</v>
       </c>
       <c r="M77" s="4" t="n">
-        <v>0.545584466835262</v>
+        <v>0.5455844668352621</v>
       </c>
       <c r="N77" s="4" t="n">
-        <v>5.381952968235262</v>
+        <v>1.379393006835262</v>
       </c>
       <c r="O77" s="4" t="n">
         <v>37.26756821176219</v>
@@ -6491,13 +6491,13 @@
         <v>1.983082073733752</v>
       </c>
       <c r="L78" s="4" t="n">
-        <v>4.963641356700001</v>
+        <v>0.8557508699999998</v>
       </c>
       <c r="M78" s="4" t="n">
-        <v>0.559941952804611</v>
+        <v>0.5599419528046111</v>
       </c>
       <c r="N78" s="4" t="n">
-        <v>5.523583309504613</v>
+        <v>1.415692822804611</v>
       </c>
       <c r="O78" s="4" t="n">
         <v>37.18411933472532</v>
@@ -6568,13 +6568,13 @@
         <v>2.033930332034616</v>
       </c>
       <c r="L79" s="4" t="n">
-        <v>5.090914212</v>
+        <v>0.8776932000000001</v>
       </c>
       <c r="M79" s="4" t="n">
-        <v>0.5742994387739599</v>
+        <v>0.5742994387739601</v>
       </c>
       <c r="N79" s="4" t="n">
-        <v>5.665213650773961</v>
+        <v>1.45199263877396</v>
       </c>
       <c r="O79" s="4" t="n">
         <v>37.1036132656314</v>
@@ -6645,13 +6645,13 @@
         <v>2.084778590335482</v>
       </c>
       <c r="L80" s="4" t="n">
-        <v>5.2181870673</v>
+        <v>0.8996355300000001</v>
       </c>
       <c r="M80" s="4" t="n">
-        <v>0.5886569247433089</v>
+        <v>0.5886569247433091</v>
       </c>
       <c r="N80" s="4" t="n">
-        <v>5.806843992043309</v>
+        <v>1.488292454743309</v>
       </c>
       <c r="O80" s="4" t="n">
         <v>37.02588687723707</v>
@@ -6722,13 +6722,13 @@
         <v>2.135626848636347</v>
       </c>
       <c r="L81" s="4" t="n">
-        <v>5.345459922599999</v>
+        <v>0.9215778600000001</v>
       </c>
       <c r="M81" s="4" t="n">
-        <v>0.6030144107126579</v>
+        <v>0.603014410712658</v>
       </c>
       <c r="N81" s="4" t="n">
-        <v>5.948474333312657</v>
+        <v>1.524592270712658</v>
       </c>
       <c r="O81" s="4" t="n">
         <v>36.95078944662159</v>
@@ -6799,13 +6799,13 @@
         <v>20.27165667754279</v>
       </c>
       <c r="L82" s="4" t="n">
-        <v>3.0848229608</v>
+        <v>0.7976458399999997</v>
       </c>
       <c r="M82" s="4" t="n">
         <v>0.2424819852601164</v>
       </c>
       <c r="N82" s="4" t="n">
-        <v>3.327304946060116</v>
+        <v>1.040127825260116</v>
       </c>
       <c r="O82" s="4" t="n">
         <v>35.36190296963254</v>
@@ -6876,13 +6876,13 @@
         <v>20.80512132695181</v>
       </c>
       <c r="L83" s="4" t="n">
-        <v>3.1660025124</v>
+        <v>0.8186365199999999</v>
       </c>
       <c r="M83" s="4" t="n">
         <v>0.2488630901353827</v>
       </c>
       <c r="N83" s="4" t="n">
-        <v>3.414865602535383</v>
+        <v>1.067499610135382</v>
       </c>
       <c r="O83" s="4" t="n">
         <v>35.30084640691653</v>
@@ -6953,13 +6953,13 @@
         <v>21.33858597636083</v>
       </c>
       <c r="L84" s="4" t="n">
-        <v>3.247182064</v>
+        <v>0.8396271999999998</v>
       </c>
       <c r="M84" s="4" t="n">
         <v>0.2552441950106489</v>
       </c>
       <c r="N84" s="4" t="n">
-        <v>3.502426259010648</v>
+        <v>1.094871395010649</v>
       </c>
       <c r="O84" s="4" t="n">
         <v>35.24208470625515</v>
@@ -7030,13 +7030,13 @@
         <v>21.87205062576984</v>
       </c>
       <c r="L85" s="4" t="n">
-        <v>3.3283616156</v>
+        <v>0.8606178799999999</v>
       </c>
       <c r="M85" s="4" t="n">
-        <v>0.261625299885915</v>
+        <v>0.2616252998859151</v>
       </c>
       <c r="N85" s="4" t="n">
-        <v>3.589986915485915</v>
+        <v>1.122243179885915</v>
       </c>
       <c r="O85" s="4" t="n">
         <v>35.185477643441</v>
@@ -7107,13 +7107,13 @@
         <v>22.40551527517886</v>
       </c>
       <c r="L86" s="4" t="n">
-        <v>3.4095411672</v>
+        <v>0.8816085599999995</v>
       </c>
       <c r="M86" s="4" t="n">
         <v>0.2680064047611813</v>
       </c>
       <c r="N86" s="4" t="n">
-        <v>3.677547571961181</v>
+        <v>1.149614964761181</v>
       </c>
       <c r="O86" s="4" t="n">
         <v>35.13089643054814</v>
@@ -7184,13 +7184,13 @@
         <v>6.47404263181796</v>
       </c>
       <c r="L87" s="4" t="n">
-        <v>3.690713501</v>
+        <v>0.8317420999999996</v>
       </c>
       <c r="M87" s="4" t="n">
         <v>0.3637229778901746</v>
       </c>
       <c r="N87" s="4" t="n">
-        <v>4.054436478890175</v>
+        <v>1.195465077890174</v>
       </c>
       <c r="O87" s="4" t="n">
         <v>36.13395562124524</v>
@@ -7261,13 +7261,13 @@
         <v>6.64441217476054</v>
       </c>
       <c r="L88" s="4" t="n">
-        <v>3.7878375405</v>
+        <v>0.8536300499999996</v>
       </c>
       <c r="M88" s="4" t="n">
         <v>0.373294635203074</v>
       </c>
       <c r="N88" s="4" t="n">
-        <v>4.161132175703074</v>
+        <v>1.226924685203074</v>
       </c>
       <c r="O88" s="4" t="n">
         <v>36.06323818839171</v>
@@ -7338,13 +7338,13 @@
         <v>6.814781717703118</v>
       </c>
       <c r="L89" s="4" t="n">
-        <v>3.88496158</v>
+        <v>0.8755179999999998</v>
       </c>
       <c r="M89" s="4" t="n">
         <v>0.3828662925159733</v>
       </c>
       <c r="N89" s="4" t="n">
-        <v>4.267827872515973</v>
+        <v>1.258384292515973</v>
       </c>
       <c r="O89" s="4" t="n">
         <v>35.99514020443488</v>
@@ -7415,13 +7415,13 @@
         <v>6.985151260645694</v>
       </c>
       <c r="L90" s="4" t="n">
-        <v>3.982085619499999</v>
+        <v>0.8974059500000001</v>
       </c>
       <c r="M90" s="4" t="n">
-        <v>0.3924379498288725</v>
+        <v>0.3924379498288726</v>
       </c>
       <c r="N90" s="4" t="n">
-        <v>4.374523569328872</v>
+        <v>1.289843899828873</v>
       </c>
       <c r="O90" s="4" t="n">
         <v>35.92950818624321</v>
@@ -7492,13 +7492,13 @@
         <v>7.155520803588272</v>
       </c>
       <c r="L91" s="4" t="n">
-        <v>4.079209659</v>
+        <v>0.9192938999999997</v>
       </c>
       <c r="M91" s="4" t="n">
         <v>0.4020096071417719</v>
       </c>
       <c r="N91" s="4" t="n">
-        <v>4.481219266141772</v>
+        <v>1.321303507141772</v>
       </c>
       <c r="O91" s="4" t="n">
         <v>35.86620051569899</v>
@@ -7569,13 +7569,13 @@
         <v>2.961642481844354</v>
       </c>
       <c r="L92" s="4" t="n">
-        <v>4.296604041199999</v>
+        <v>0.8658383599999996</v>
       </c>
       <c r="M92" s="4" t="n">
         <v>0.4849639705202328</v>
       </c>
       <c r="N92" s="4" t="n">
-        <v>4.781568011720232</v>
+        <v>1.350802330520232</v>
       </c>
       <c r="O92" s="4" t="n">
         <v>36.68495957185565</v>
@@ -7646,13 +7646,13 @@
         <v>3.03958044189289</v>
       </c>
       <c r="L93" s="4" t="n">
-        <v>4.4096725686</v>
+        <v>0.8886235799999994</v>
       </c>
       <c r="M93" s="4" t="n">
         <v>0.4977261802707653</v>
       </c>
       <c r="N93" s="4" t="n">
-        <v>4.907398748870765</v>
+        <v>1.386349760270765</v>
       </c>
       <c r="O93" s="4" t="n">
         <v>36.60778341688533</v>
@@ -7723,13 +7723,13 @@
         <v>3.117518401941425</v>
       </c>
       <c r="L94" s="4" t="n">
-        <v>4.522741095999999</v>
+        <v>0.9114087999999998</v>
       </c>
       <c r="M94" s="4" t="n">
         <v>0.5104883900212978</v>
       </c>
       <c r="N94" s="4" t="n">
-        <v>5.033229486021296</v>
+        <v>1.421897190021298</v>
       </c>
       <c r="O94" s="4" t="n">
         <v>36.53340348017442</v>
@@ -7800,13 +7800,13 @@
         <v>3.195456361989962</v>
       </c>
       <c r="L95" s="4" t="n">
-        <v>4.635809623399999</v>
+        <v>0.9341940199999997</v>
       </c>
       <c r="M95" s="4" t="n">
-        <v>0.5232505997718301</v>
+        <v>0.5232505997718302</v>
       </c>
       <c r="N95" s="4" t="n">
-        <v>5.15906022317183</v>
+        <v>1.45744461977183</v>
       </c>
       <c r="O95" s="4" t="n">
         <v>36.46166111116385</v>
@@ -7877,13 +7877,13 @@
         <v>3.273394322038497</v>
       </c>
       <c r="L96" s="4" t="n">
-        <v>4.7488781508</v>
+        <v>0.9569792399999995</v>
       </c>
       <c r="M96" s="4" t="n">
         <v>0.5360128095223626</v>
       </c>
       <c r="N96" s="4" t="n">
-        <v>5.284890960322362</v>
+        <v>1.492992049522362</v>
       </c>
       <c r="O96" s="4" t="n">
         <v>36.39240967505654</v>
@@ -7954,13 +7954,13 @@
         <v>1.653630323944945</v>
       </c>
       <c r="L97" s="4" t="n">
-        <v>4.902494581399999</v>
+        <v>0.8999346199999995</v>
       </c>
       <c r="M97" s="4" t="n">
         <v>0.606204963150291</v>
       </c>
       <c r="N97" s="4" t="n">
-        <v>5.50869954455029</v>
+        <v>1.50613958315029</v>
       </c>
       <c r="O97" s="4" t="n">
         <v>37.09111197460639</v>
@@ -8031,13 +8031,13 @@
         <v>1.69714691141718</v>
       </c>
       <c r="L98" s="4" t="n">
-        <v>5.0315075967</v>
+        <v>0.9236171099999995</v>
       </c>
       <c r="M98" s="4" t="n">
         <v>0.6221577253384566</v>
       </c>
       <c r="N98" s="4" t="n">
-        <v>5.653665322038457</v>
+        <v>1.545774835338456</v>
       </c>
       <c r="O98" s="4" t="n">
         <v>37.00950076000471</v>
@@ -8108,13 +8108,13 @@
         <v>1.740663498889416</v>
       </c>
       <c r="L99" s="4" t="n">
-        <v>5.160520612</v>
+        <v>0.9472995999999997</v>
       </c>
       <c r="M99" s="4" t="n">
         <v>0.6381104875266221</v>
       </c>
       <c r="N99" s="4" t="n">
-        <v>5.798631099526622</v>
+        <v>1.585410087526622</v>
       </c>
       <c r="O99" s="4" t="n">
         <v>36.93079120095626</v>
@@ -8185,13 +8185,13 @@
         <v>1.784180086361651</v>
       </c>
       <c r="L100" s="4" t="n">
-        <v>5.2895336273</v>
+        <v>0.9709820899999997</v>
       </c>
       <c r="M100" s="4" t="n">
-        <v>0.6540632497147877</v>
+        <v>0.6540632497147878</v>
       </c>
       <c r="N100" s="4" t="n">
-        <v>5.943596877014787</v>
+        <v>1.625045339714787</v>
       </c>
       <c r="O100" s="4" t="n">
         <v>36.85482158101389</v>
@@ -8262,13 +8262,13 @@
         <v>1.827696673833886</v>
       </c>
       <c r="L101" s="4" t="n">
-        <v>5.418546642600001</v>
+        <v>0.9946645799999997</v>
       </c>
       <c r="M101" s="4" t="n">
         <v>0.6700160119029531</v>
       </c>
       <c r="N101" s="4" t="n">
-        <v>6.088562654502954</v>
+        <v>1.664680591902953</v>
       </c>
       <c r="O101" s="4" t="n">
         <v>36.7814424325773</v>

</xml_diff>